<commit_message>
Remove optional attachment URL in templates
</commit_message>
<xml_diff>
--- a/web/static/templates/httpsms-bulk.xlsx
+++ b/web/static/templates/httpsms-bulk.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Arnold\Work\NdoleStudio\httpsms.com\web\static\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B440C98-E1CB-43F3-9EF7-15E26C17E41D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B6E92B1-2F21-44BE-AEC5-4C0A2FC1EE92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1140" yWindow="0" windowWidth="25780" windowHeight="20880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>FromPhoneNumber</t>
   </si>
@@ -34,9 +34,6 @@
     <t>SendTime(optional)</t>
   </si>
   <si>
-    <t>AttachmentURLs(optional)</t>
-  </si>
-  <si>
     <t>This is a sample text message1</t>
   </si>
   <si>
@@ -44,9 +41,6 @@
   </si>
   <si>
     <t>2023-11-11T02:10:01</t>
-  </si>
-  <si>
-    <t>https://placehold.co/600x400/png</t>
   </si>
 </sst>
 </file>
@@ -339,9 +333,7 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
+      <c r="E1" s="1"/>
     </row>
     <row r="2" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1">
@@ -351,11 +343,9 @@
         <v>18005550100</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>8</v>
-      </c>
+      <c r="E2" s="2"/>
     </row>
     <row r="3" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1">
@@ -365,10 +355,10 @@
         <v>18005550100</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
@@ -1369,9 +1359,6 @@
     <row r="999" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="1000" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="E2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
 </worksheet>

</xml_diff>